<commit_message>
Update toner configuration, review UI and submitter identity
</commit_message>
<xml_diff>
--- a/backend/data/HP_Toner_Printer_Compatibility.xlsx
+++ b/backend/data/HP_Toner_Printer_Compatibility.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E180"/>
+  <dimension ref="A1:E183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="16.1328125" customWidth="1" min="2" max="2"/>
@@ -496,7 +496,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LaserJet P1007, P1008, P1106, P1108, M1136 MFP</t>
+          <t>LaserJet P1007, P1008, P1106, P1108, M1136 MFP, LaserJet Pro MFP M126a</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>LaserJet 1010, 1012, 1015, 1018, 1020, 1022, 3015, 3050, 3052, 3055, M1005</t>
+          <t>LaserJet 1010, 1012, 1015, 1018, 1020, 1022, 3015, 3050, 3052, 3055, M1005, 3020, 3030, M1319 MFP, 1020 Plus</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LaserJet P1566, P1606dn, M1536dnf</t>
+          <t>LaserJet P1566, P1606dn, M1536dnf, P1560</t>
         </is>
       </c>
     </row>
@@ -586,17 +586,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TNB021</t>
+          <t>W1660A</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Brother</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>HL-B2000D, DCP-B7500D, DCP-B7535DW, MFC-B7715DW</t>
+          <t>Laser 1008a, 1008w, MFP 1188a,1188w</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TN2365</t>
+          <t>W1370</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Brother</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HL-L2321D, HL-L2361DN, HL-L2366DW, DCP-L2520D, DCP-L2541DW, MFC-L2701D, MFC-L2703DW</t>
+          <t>LaserJet M208, M209, MFP M233, M234</t>
         </is>
       </c>
     </row>
@@ -626,17 +626,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>W1660A</t>
+          <t>CE285A/CRG925</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>HP / Canon</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Laser 1008a, 1008w, MFP 1188a,1188w</t>
+          <t>HP LaserJet P1102, P1102w, M1130 MFP, M1132 MFP, M1210 MFP, M1212nf MFP, M1217nfw MFP, P1100, P1101 / Canon LBP6000, LBP6018, LBP6030, imageCLASS MF3010, LBP6018b, LBP6030b, LBP6030w</t>
         </is>
       </c>
     </row>
@@ -646,17 +646,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>W1370</t>
+          <t>CF283A/CRG337</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>HP / Canon</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LaserJet M208, M209, MFP M233, M234</t>
+          <t>HP LaserJet Pro M125, M127, M201, M225 / Canon imageCLASS MF211, MF215, MF216, MF229, MF212, MF217, MF226, MF232w, MF237w, MF241d, MF244dw, MF246dn, MF249dw, MF235, LBP151dw</t>
         </is>
       </c>
     </row>
@@ -666,17 +666,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CRG071</t>
+          <t>CF230A</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LBP122dw, LBP121dn, MF272dw, MF275dw</t>
+          <t>LaserJet Pro M203, M203dw, M227fdw, M227sdn</t>
         </is>
       </c>
     </row>
@@ -686,17 +686,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CE285A/CRG925</t>
+          <t>W1520A</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>HP LaserJet P1102, M1132, M1212nf / Canon LBP6000, LBP6030, MF3010</t>
+          <t>LaserJet Pro 4003, 4004, MFP4103, MFP4104</t>
         </is>
       </c>
     </row>
@@ -706,17 +706,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CF283A/CRG337</t>
+          <t>CE505A/CF280A</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>HP LaserJet Pro M125, M127, M201, M225 / Canon MF211, MF215, MF216, MF229</t>
+          <t>P2035, P2055 / LaserJet Pro 400 M401, M425</t>
         </is>
       </c>
     </row>
@@ -726,17 +726,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CF230A</t>
+          <t>CB435A</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>HP / Canon</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LaserJet Pro M203, M203dw, M227fdw, M227sdn</t>
+          <t>HP LaserJet P1005, P1006 / Canon LBP3018, LBP3108, LBP3050</t>
         </is>
       </c>
     </row>
@@ -746,17 +746,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>W1520A</t>
+          <t>CB436A</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>HP / Canon</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>LaserJet Pro 4003, 4004, MFP4103, MFP4104</t>
+          <t>HP LaserJet P1505, P1500, M1120, M1522 / Canon LBP3250</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CE505A/CF280A</t>
+          <t>CE255A</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>P2035, P2055 / LaserJet Pro 400 M401, M425</t>
+          <t>LaserJet P3015, P3010, LaserJet Enterprise 500 M521, LaserJet Enterprise 500 MFP M525</t>
         </is>
       </c>
     </row>
@@ -786,17 +786,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PC-210</t>
+          <t>CC364A</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pantum</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>P2200, P2207, P2500, M6500, M6550</t>
+          <t>LaserJet P4015, P4515, P4014</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PC-208</t>
+          <t>Q7516A</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pantum</t>
+          <t>HP / Canon</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>P2508, M6508, M6558</t>
+          <t>HP LaserJet 5200 / Canon LBP3500, LBP3900, LBP3950, LBP3970</t>
         </is>
       </c>
     </row>
@@ -826,17 +826,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>TL-412</t>
+          <t>CF279A</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Pantum</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BP5100, BM5100</t>
+          <t>LaserJet Pro M12a, M12w, LaserJet Pro MFP M26a, M26nw</t>
         </is>
       </c>
     </row>
@@ -846,17 +846,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>TL-425</t>
+          <t>CF244A</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pantum</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>BP5100DN, BM5100ADN</t>
+          <t>LaserJet Pro M15a, M15w, LaserJet Pro MFP M28a, M28w</t>
         </is>
       </c>
     </row>
@@ -866,17 +866,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TL-5120</t>
+          <t>CF217A</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Pantum</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>BP5100 series, BM5100 series</t>
+          <t>LaserJet Pro M102, LaserJet Pro MFP M130</t>
         </is>
       </c>
     </row>
@@ -886,17 +886,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CB435A</t>
+          <t>CF226A</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>HP LaserJet P1005, P1006 / Canon LBP3018, LBP3108, LBP3050</t>
+          <t>LaserJet Pro M402, LaserJet Pro MFP M426</t>
         </is>
       </c>
     </row>
@@ -906,17 +906,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CB436A</t>
+          <t>CF228A</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>HP LaserJet P1505, M1120, M1522, P1500 / Canon LBP3250</t>
+          <t>LaserJet Pro M403, LaserJet Pro MFP M427</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CE255A</t>
+          <t>CF276A</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>LaserJet P3015, P3010</t>
+          <t>LaserJet Pro M304, M404, LaserJet Pro MFP M428</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CC364A</t>
+          <t>CZ192A</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>LaserJet P4015, P4515, P4014</t>
+          <t>LaserJet Pro M435nw, M701, M706</t>
         </is>
       </c>
     </row>
@@ -966,17 +966,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Q7516A</t>
+          <t>CF287A</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>HP LaserJet 5200 / Canon LBP3500, LBP3900, LBP3950, LBP3970</t>
+          <t>LaserJet Enterprise M501, M506, LaserJet Enterprise MFP M527, LaserJet Enterprise M505x</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CF279A</t>
+          <t>CF237A</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>LaserJet Pro M12a, M12w, LaserJet Pro MFP M26a, M26nw</t>
+          <t>LaserJet Enterprise M607, M608, M609, LaserJet Enterprise MFP M631, M632, M633</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CF244A</t>
+          <t>W1500A</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>LaserJet Pro M15a, M15w, LaserJet Pro MFP M28a, M28w</t>
+          <t>LaserJet M111a, M111w, LaserJet MFP M141a, M141w</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CF217A</t>
+          <t>W1360A</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>LaserJet Pro M102, LaserJet Pro MFP M130</t>
+          <t>LaserJet M211d, M211dw, LaserJet MFP M232, M233, M234, M236</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CF226A</t>
+          <t>W1103A</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>LaserJet Pro M402, LaserJet Pro MFP M426</t>
+          <t>LaserJet Neverstop / Tank 1000, 1005, 1200, 1202</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CF228A</t>
+          <t>W1530A</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>LaserJet Pro M403, LaserJet Pro MFP M427</t>
+          <t>LaserJet Tank 1502, 1504, 2502, 2506, 2602, 2606</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CF276A</t>
+          <t>CE310A/CE311A/CE312A/CE313A</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>LaserJet Pro M304, M404, LaserJet Pro MFP M428</t>
+          <t>Color LaserJet CP1025, Color LaserJet MFP M175, M275</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CZ192A</t>
+          <t>CB540A/CB541A/CB542A/CB543A</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LaserJet Pro M435nw, M701, M706</t>
+          <t>Color LaserJet CP1215, CP1515, CP1518, CM1312</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CF287A</t>
+          <t>CC530A/CC531A/CC532A/CC533A</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LaserJet Enterprise M501, M506, LaserJet Enterprise MFP M527, LaserJet Enterprise M505x</t>
+          <t>Color LaserJet CP2025, CM2320, CP2020</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CF237A</t>
+          <t>CF510A/CF511A/CF512A/CF513A</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LaserJet Enterprise M607, M608, M609</t>
+          <t>Color LaserJet Pro M154, Color LaserJet Pro MFP M180, M181</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>W1500A</t>
+          <t>CF400A/CF401A/CF402A/CF403A</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>LaserJet M111a, M111w, LaserJet MFP M141a, M141w</t>
+          <t>Color LaserJet Pro M252, Color LaserJet Pro MFP M277</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>W1360A</t>
+          <t>CF540A/CF541A/CF542A/CF543A</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>LaserJet M211d, M211dw, LaserJet MFP M232, M233, M234, M236</t>
+          <t>Color LaserJet Pro M254, Color LaserJet Pro MFP M280, M281</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>W1103A</t>
+          <t>W2110A/W2111A/W2112A/W2113A</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>LaserJet Neverstop / Tank 1000, 1005, 1200, 1202</t>
+          <t>Color LaserJet Pro M255, Color LaserJet Pro MFP M282, M283</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>W1530A</t>
+          <t>CF410A/CF411A/CF412A/CF413A</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>LaserJet Tank 1502, 1504, 2502, 2506, 2602, 2606</t>
+          <t>Color LaserJet Pro M452, Color LaserJet Pro MFP M477, M377</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CE310A/CE311A/CE312A/CE313A</t>
+          <t>W2030A/W2031A/W2032A/W2033A</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Color LaserJet CP1025, Color LaserJet MFP M175, M275</t>
+          <t>Color LaserJet Pro M454, Color LaserJet Pro MFP M479</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CB540A/CB541A/CB542A/CB543A</t>
+          <t>W2070A/W2071A/W2072A/W2073A</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Color LaserJet CP1515, CP1525, CM1312, CP1215</t>
+          <t>Color Laser 150a, 150nw, Color Laser MFP 178nw, 179fnw</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CC530A/CC531A/CC532A/CC533A</t>
+          <t>Q2624A</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Color LaserJet CP2025, CM2320, CP2020</t>
+          <t>LaserJet 1150, 1150N, 1300, 1300N, 1300XI, 3300 MFP, 3320n, 3320 MFP, 3330 MFP</t>
         </is>
       </c>
     </row>
@@ -1306,17 +1306,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CF510A/CF511A/CF512A/CF513A</t>
+          <t>C7115A</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>HP / Canon</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro M154, Color LaserJet Pro MFP M180, M181</t>
+          <t>HP LaserJet 1000, 1005, 1200, 1200N, 1200SE, 1220, 1220SE / Canon LBP1210</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CF400A/CF401A/CF402A/CF403A</t>
+          <t>CF228X</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro M252, Color LaserJet Pro MFP M277</t>
+          <t>LaserJet Pro M403, LaserJet Pro MFP M427</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CF540A/CF541A/CF542A/CF543A</t>
+          <t>C4129X</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro M254, Color LaserJet Pro MFP M280, M281</t>
+          <t>LaserJet 5000, 5100</t>
         </is>
       </c>
     </row>
@@ -1366,17 +1366,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>W2110A/W2111A/W2112A/W2113A</t>
+          <t>Q5949A</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>HP / Canon</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro M255, Color LaserJet Pro MFP M282, M283</t>
+          <t>HP LaserJet 1160, 1320, 3390, 3392 / Canon LBP3300, LBP3310, LBP3360, LBP3370</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CF410A/CF411A/CF412A/CF413A</t>
+          <t>Q7551A</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro M452, Color LaserJet Pro MFP M477, M377</t>
+          <t>LaserJet P3005, M3027, M3035</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>W2030A/W2031A/W2032A/W2033A</t>
+          <t>Q7570A</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro M454, Color LaserJet Pro MFP M479</t>
+          <t>LaserJet M5025, M5035</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>W2070A/W2071A/W2072A/W2073A</t>
+          <t>CF280X</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Color Laser 150a, 150nw, Color Laser MFP 178nw, 179fnw</t>
+          <t>LaserJet Pro 400 M401, LaserJet Pro 400 MFP M425</t>
         </is>
       </c>
     </row>
@@ -1446,17 +1446,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CRG303</t>
+          <t>CF247A</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>LBP2900, LBP3000</t>
+          <t>LaserJet Pro M15a, M16, LaserJet Pro MFP M28a</t>
         </is>
       </c>
     </row>
@@ -1466,17 +1466,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CRG125</t>
+          <t>CF277X</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>LBP6000, LBP6000B, LBP6018, LBP6018L, LBP6018W, LBP6020, LBP6020B, LBP6030, LBP6030w, LBP6040, imageCLASS MF3010</t>
+          <t>LaserJet Pro MFP M429</t>
         </is>
       </c>
     </row>
@@ -1486,17 +1486,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TN2260</t>
+          <t>CF281A</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Brother / Konica Minolta</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Brother HL-2130, HL-2240D, HL-2250DN, DCP-7060D, DCP-7065DN, MFC-7360, MFC-7860DW, FAX-2840, DCP-7055 / Konica Minolta 1580</t>
+          <t>LaserJet Enterprise M604n, M604dn, M605n, M605x, M605dn, M606x, M606dn, LaserJet Enterprise MFP M630f, M630z, M630dn, M630h</t>
         </is>
       </c>
     </row>
@@ -1506,17 +1506,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MLT-D111S</t>
+          <t>CF281X</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Xpress SL-M2020, SL-M2020W, SL-M2021, SL-M2021W, SL-M2022, SL-M2022W, SL-M2024, SL-M2026, SL-M2026W, SL-M2070, SL-M2070W, SL-M2070F, SL-M2070FW, SL-M2071, SL-M2071W, SL-M2071FH, SL-M2074FW, SL-M2077, SL-M2078, SL-M2078F, SL-M2078FW</t>
+          <t>LaserJet Enterprise M605n, M605x, M605dn, M606x, M606dn, LaserJet Enterprise MFP M630f, M630z, M630dn, M630h</t>
         </is>
       </c>
     </row>
@@ -1526,17 +1526,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TK-160</t>
+          <t>CF287X</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>FS-1120D, FS-1120DN, ECOSYS P2035d, P2035dn</t>
+          <t>LaserJet Enterprise M501, M505x, M506, LaserJet Enterprise MFP M527</t>
         </is>
       </c>
     </row>
@@ -1546,17 +1546,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TK-1122</t>
+          <t>CF214X</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>FS-1060DN, FS-1025MFP, FS-1125MFP</t>
+          <t>LaserJet Enterprise 700 M712, LaserJet Enterprise 700 MFP M725</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>TK-1134</t>
+          <t>CF218A</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>FS-1030MFP, FS-1130MFP, ECOSYS M2030dn, M2530dn</t>
+          <t>LaserJet Pro M102, M104, LaserJet Pro MFP M130, M132</t>
         </is>
       </c>
     </row>
@@ -1586,17 +1586,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>TK-1140</t>
+          <t>CF233A</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>FS-1035MFP, FS-1135MFP, ECOSYS M2035dn, M2535dn</t>
+          <t>LaserJet M106, M106w, LaserJet MFP M134, M134a, M134fn</t>
         </is>
       </c>
     </row>
@@ -1606,17 +1606,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TK-1144</t>
+          <t>CF237X</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>FS-1035MFP, FS-1135MFP, ECOSYS M2035dn, M2535dn</t>
+          <t>LaserJet Enterprise M608, M609, LaserJet Enterprise MFP M631, M632, M633</t>
         </is>
       </c>
     </row>
@@ -1626,17 +1626,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>TK-1170</t>
+          <t>CF256A</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ECOSYS M2040dn, M2540dn, M2640idw</t>
+          <t>LaserJet MFP M436, M433</t>
         </is>
       </c>
     </row>
@@ -1646,17 +1646,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TK-3100</t>
+          <t>CF256X</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>FS-2100D, FS-2100DN, FS-4100DN, FS-4200DN, FS-4300DN, ECOSYS M3040dn, M3540dn</t>
+          <t>LaserJet MFP M436nda, M436</t>
         </is>
       </c>
     </row>
@@ -1666,17 +1666,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TN1020</t>
+          <t>C8543X</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Brother</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>HL-1111, HL-1201, HL-1211W, DCP-1511, DCP-1514, DCP-1601, DCP-1616NW, MFC-1811, MFC-1814, MFC-1911NW</t>
+          <t>LaserJet 9000, 9040, 9050, M9040, M9050, M9059</t>
         </is>
       </c>
     </row>
@@ -1686,17 +1686,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TN2150</t>
+          <t>W1580X</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Brother / Ricoh</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Brother DCP-7030, DCP-7040, DCP-7045N, HL-2140, HL-2025, HL-2150N, HL-2170W, MFC-7440N, MFC-7840W, MFC-7340, MFC-7345DN, MFC-7320, MFC-7345N / Ricoh SP 1200</t>
+          <t>LaserJet Pro 3002dn, 3002dw, MFP 3102fdn, MFP 3102fdw</t>
         </is>
       </c>
     </row>
@@ -1706,17 +1706,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TN3185</t>
+          <t>CF325X</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Brother</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>HL-5240, HL-5250, HL-5270, MFC-8460, MFC-8860, HL-5340D, HL-5350DN, HL-5380DN, HL-5370W, MFC-8380DN, MFC-8880DN, HL-5340, HL-5350, HL-5370, HL-5370DW, DCP-8070, DCP-8080, DCP-8085, MFC-8370, MFC-8380, MFC-8480, MFC-8680, MFC-8690, MFC-8880, MFC-8890</t>
+          <t>LaserJet Enterprise M800, M806, M806dn, LaserJet Enterprise MFP M830z</t>
         </is>
       </c>
     </row>
@@ -1726,17 +1726,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>TN3350</t>
+          <t>CF289A</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Brother</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>HL-5440, DCP-8110DN, DCP-8150DN, DCP-8250DN, MFC-8510DN, MFC-8910DW</t>
+          <t>LaserJet Enterprise M507, LaserJet Enterprise MFP M528</t>
         </is>
       </c>
     </row>
@@ -1746,17 +1746,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>TN3448</t>
+          <t>CE390X</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Brother</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>HL-5000, HL-5100, HL-6200, HL-6900, MFC-5900, MFC-5700</t>
+          <t>LaserJet P4014, P4015, P4515, LaserJet Enterprise M601, M602, M603, M4555</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1766,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TN3478</t>
+          <t>CE390A</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Brother</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>HL-5000, HL-5100, HL-6200, HL-6900, MFC-5900, MFC-5700</t>
+          <t>LaserJet P4014, P4015, P4515, LaserJet Enterprise M601, M602, M603, M4555</t>
         </is>
       </c>
     </row>
@@ -1786,15 +1786,19 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TN2465</t>
+          <t>W1004AC</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Brother</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Laser MFP 131a, Laser 103a</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1802,17 +1806,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TN261BK/TN261C/TN261Y/TN261M</t>
+          <t>W1335X</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Brother</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>HL-3140CW, HL-3150CDN, HL-3150CDW, HL-3170CDW, MFC-9130CW, MFC-9140CDN, MFC-9330CDW, MFC-9340CDW</t>
+          <t>LaserJet MFP M438, M442dn, M443</t>
         </is>
       </c>
     </row>
@@ -1822,17 +1826,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>TN267BK/TN267C/TN267Y/TN267M</t>
+          <t>W1370X</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Brother</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>HL-L3230CDN, MFC-L3750</t>
+          <t>LaserJet M208, M209, M211d, LaserJet MFP M232, M233, M234, M236</t>
         </is>
       </c>
     </row>
@@ -1842,17 +1846,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>CRG319</t>
+          <t>CE320A/CE321A/CE322A/CE323A</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>LBP6300, LBP6650, imageCLASS MF416</t>
+          <t>Color LaserJet CP1525, CM1415</t>
         </is>
       </c>
     </row>
@@ -1862,17 +1866,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>CRG319H</t>
+          <t>CF210A/CF211A/CF212A/CF213A</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>LBP6300, LBP6650, LBP251, LBP252, LBP253, imageCLASS MF414, MF416</t>
+          <t>Color LaserJet Pro 200</t>
         </is>
       </c>
     </row>
@@ -1882,17 +1886,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CRG039</t>
+          <t>CF350A/CF351A/CF352A/CF353A</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>LBP351dn, LBP351x, LBP351xz, LBP352dn, LBP352x, LBP352i, LBP351i, LBP352xz</t>
+          <t>Color LaserJet Pro MFP M176, M177</t>
         </is>
       </c>
     </row>
@@ -1902,17 +1906,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CRG039H</t>
+          <t>CE410A/CE411A/CE412A/CE413A</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>LBP351dn, LBP351x, LBP351xz, LBP352dn, LBP352x, LBP352i, LBP351i, LBP352xz</t>
+          <t>Color LaserJet Pro 300 M351, Color LaserJet Pro 300 MFP M375nw, Color LaserJet Pro 400 M451nw, M451dn, M451dw, Color LaserJet Pro 400 MFP M475dn, M475dw</t>
         </is>
       </c>
     </row>
@@ -1922,17 +1926,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>CRG045BK/CRG045C/CRG045Y/CRG045M</t>
+          <t>CF380A/CF381A/CF382A/CF383A</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>imageCLASS MF634Cdw, MF632Cdw, LBP612Cdw</t>
+          <t>Color LaserJet Pro MFP M476dn</t>
         </is>
       </c>
     </row>
@@ -1942,17 +1946,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CRG046BK/CRG046C/CRG046Y/CRG046M</t>
+          <t>CF500A/CF501A/CF502A/CF503A</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>imageCLASS MF733Cdw, MF731Cdw, MF735Cd</t>
+          <t>Color LaserJet Pro M254, Color LaserJet Pro MFP M280, M281</t>
         </is>
       </c>
     </row>
@@ -1962,17 +1966,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CRG050</t>
+          <t>Q6000A/Q6001A/Q6002A/Q6003A</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>LBP910 Series, LBP913, imageCLASS MF910 Series, imageCLASS MF913</t>
+          <t>Color LaserJet 1600, 2600n, 2605, 2605dn, 2605dtn, CM1017, CM1015</t>
         </is>
       </c>
     </row>
@@ -1982,17 +1986,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>CRG052</t>
+          <t>CE250A/CE251A/CE252A/CE253A</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>LBP214dw, LBP215dw, imageCLASS MF424dw, MF426dw, MF429dw</t>
+          <t>Color LaserJet CP3525, CP3525n, CP3525dn, CM3530, CM3530fs</t>
         </is>
       </c>
     </row>
@@ -2002,17 +2006,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>CRG054BK/CRG054C/CRG054Y/CRG054M</t>
+          <t>CE400A/CE401A/CE402A/CE403A</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>imageCLASS MF642</t>
+          <t>Color LaserJet Enterprise 500 M551n, M551dn, M551xh</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2026,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CRG057</t>
+          <t>CE260A/CE261A/CE262A/CE263A</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>LBP220, LBP223dw, LBP226dw, LBP227dw, LBP228x, LBP228dw, imageCLASS MF440, MF443dw, MF445dw, MF446x, MF448dw, MF449x, MF449dw</t>
+          <t>Color LaserJet CP4025, CP4520, CM4540</t>
         </is>
       </c>
     </row>
@@ -2042,17 +2046,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CRG041</t>
+          <t>CE270A/CE271A/CE272A/CE273A</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>imageCLASS LBP312x, LBP312dn</t>
+          <t>Color LaserJet CP5525n, CP5525dn, CP5525xh</t>
         </is>
       </c>
     </row>
@@ -2062,17 +2066,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>NPG-51</t>
+          <t>W2310A/W2311A/W2312A/W2313A</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>GPR-35, iR2520, iR2525, iR2530</t>
+          <t>Color LaserJet Pro M155, Color LaserJet Pro MFP M182, M183</t>
         </is>
       </c>
     </row>
@@ -2082,17 +2086,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>NPG-59</t>
+          <t>W2040A/W2041A/W2042A/W2043A</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>iR2002, iR2202, iR2204, iR2004</t>
+          <t>Color LaserJet Pro M454, Color LaserJet Pro MFP M479</t>
         </is>
       </c>
     </row>
@@ -2102,17 +2106,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>NPG-28</t>
+          <t>W2090A/W2091A/W2092A/W2093A</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>iR2318, iR2018, iR2422, iR2420</t>
+          <t>Color Laser MFP 178nw, Color Laser 150a, 150nw</t>
         </is>
       </c>
     </row>
@@ -2122,17 +2126,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>NPG-84</t>
+          <t>CE740A/CE741A/CE742A/CE743A</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>iR2625, iR2645</t>
+          <t>Color LaserJet CP5225, CP5225n, CP5225dn</t>
         </is>
       </c>
     </row>
@@ -2142,17 +2146,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>1130</t>
+          <t>CRG071</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>1130</t>
+          <t>LBP122dw, LBP121dn, MF272dw, MF275dw</t>
         </is>
       </c>
     </row>
@@ -2162,17 +2166,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Q2624A</t>
+          <t>CRG303</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>HP LaserJet 1000, 1005, 1200N, 1200SE, 1220, 1220SE, LaserJet 3300 MFP, LaserJet 3320n, LaserJet 3320 MFP, LaserJet 3330 MFP, LaserJet 1300, 1300N, 1300XI, 1150, 1150N / Canon LBP1210</t>
+          <t>LBP2900, LBP3000</t>
         </is>
       </c>
     </row>
@@ -2182,17 +2186,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>C7115A</t>
+          <t>CRG125</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>HP LaserJet 1000, 1200, 1220 / Canon LBP1210</t>
+          <t>LBP6000, LBP6000B, LBP6018, LBP6018L, LBP6018W, LBP6020, LBP6020B, LBP6030, LBP6030w, LBP6040, imageCLASS MF3010</t>
         </is>
       </c>
     </row>
@@ -2202,17 +2206,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>CF228X</t>
+          <t>CRG319</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>LaserJet Pro M403, LaserJet Pro MFP M427</t>
+          <t>LBP6300, LBP6650, imageCLASS MF416</t>
         </is>
       </c>
     </row>
@@ -2222,17 +2226,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>C4129X</t>
+          <t>CRG319H</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>LaserJet 5000, 5100</t>
+          <t>LBP6300, LBP6650, LBP251, LBP252, LBP253, imageCLASS MF414, MF416</t>
         </is>
       </c>
     </row>
@@ -2242,17 +2246,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Q5949A</t>
+          <t>CRG039</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>HP LaserJet 1160, 1320, P2015, P2014 / Canon LBP3300, LBP3360, LBP3310, LBP3370</t>
+          <t>LBP351dn, LBP351x, LBP351xz, LBP352dn, LBP352x, LBP352i, LBP351i, LBP352xz</t>
         </is>
       </c>
     </row>
@@ -2262,17 +2266,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Q7551A</t>
+          <t>CRG039H</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>LaserJet P3005, M3027, M3035</t>
+          <t>LBP351dn, LBP351x, LBP351xz, LBP352dn, LBP352x, LBP352i, LBP351i, LBP352xz</t>
         </is>
       </c>
     </row>
@@ -2282,17 +2286,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Q7570A</t>
+          <t>CRG045BK/CRG045C/CRG045Y/CRG045M</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>LaserJet M5025, M5035</t>
+          <t>imageCLASS MF634Cdw, MF632Cdw, LBP612Cdw</t>
         </is>
       </c>
     </row>
@@ -2302,17 +2306,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CF280X</t>
+          <t>CRG046BK/CRG046C/CRG046Y/CRG046M</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>HP LaserJet Pro 400 M401, LaserJet Pro 400 MFP M425 / Canon 3196H</t>
+          <t>imageCLASS MF733Cdw, MF731Cdw, MF735Cd</t>
         </is>
       </c>
     </row>
@@ -2322,17 +2326,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>CF247A</t>
+          <t>CRG050</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>LaserJet Pro M15a, M16, LaserJet Pro MFP M28a</t>
+          <t>LBP910 Series, LBP913, imageCLASS MF910 Series, imageCLASS MF913</t>
         </is>
       </c>
     </row>
@@ -2342,17 +2346,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>CF277X</t>
+          <t>CRG052</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>LaserJet Pro MFP M429</t>
+          <t>LBP214dw, LBP215dw, imageCLASS MF424dw, MF426dw, MF429dw</t>
         </is>
       </c>
     </row>
@@ -2362,17 +2366,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>CF281A</t>
+          <t>CRG054BK/CRG054C/CRG054Y/CRG054M</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>LaserJet Enterprise M604n, M604dn, M605n, M605x, M605dn, M606x, M606dn, LaserJet Enterprise MFP M630f, M630z, M630dn, M630h</t>
+          <t>imageCLASS MF642</t>
         </is>
       </c>
     </row>
@@ -2382,17 +2386,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>CF281X</t>
+          <t>CRG057</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>LaserJet Enterprise M605n, M605x, M605dn, M606x, M606dn, LaserJet Enterprise MFP M630f, M630z, M630dn, M630h</t>
+          <t>LBP220, LBP223dw, LBP226dw, LBP227dw, LBP228x, LBP228dw, imageCLASS MF440, MF443dw, MF445dw, MF446x, MF448dw, MF449x, MF449dw</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2406,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>CF287X</t>
+          <t>CRG041</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>LaserJet Enterprise M501, M505x, M506, LaserJet Enterprise MFP M527</t>
+          <t>imageCLASS LBP312x, LBP312dn</t>
         </is>
       </c>
     </row>
@@ -2422,17 +2426,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>CF214X</t>
+          <t>NPG-51</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>LaserJet Enterprise 700 M712</t>
+          <t>GPR-35, iR2520, iR2525, iR2530</t>
         </is>
       </c>
     </row>
@@ -2442,17 +2446,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>CF218A</t>
+          <t>NPG-59</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>LaserJet Pro M102, M104, LaserJet Pro MFP M130, M132</t>
+          <t>iR2002, iR2202, iR2204, iR2004</t>
         </is>
       </c>
     </row>
@@ -2462,17 +2466,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>CF233A</t>
+          <t>NPG-28</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>LaserJet M106, M106w, LaserJet MFP M134, M134a, M134fn</t>
+          <t>iR2318, iR2018, iR2422, iR2420</t>
         </is>
       </c>
     </row>
@@ -2482,17 +2486,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>CF237X</t>
+          <t>NPG-84</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>LaserJet Enterprise M608, M609</t>
+          <t>iR2625, iR2645</t>
         </is>
       </c>
     </row>
@@ -2502,17 +2506,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>CF256A</t>
+          <t>TNB021</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>LaserJet MFP M436, M433</t>
+          <t>HL-B2000D, DCP-B7500D, DCP-B7535DW, MFC-B7715DW</t>
         </is>
       </c>
     </row>
@@ -2522,17 +2526,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>CF256X</t>
+          <t>TN2365</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>LaserJet MFP M436nda, M436</t>
+          <t>HL-L2321D, HL-L2361DN, HL-L2366DW, DCP-L2520D, DCP-L2541DW, MFC-L2701D, MFC-L2703DW</t>
         </is>
       </c>
     </row>
@@ -2542,17 +2546,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>C8543X</t>
+          <t>TN2260</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>LaserJet 9000, 9040, 9050, M9040, M9050, M9059</t>
+          <t>HL-2240D, HL-2250DN, DCP-7060D, DCP-7065DN, MFC-7360, MFC-7860DW, FAX-2840</t>
         </is>
       </c>
     </row>
@@ -2562,17 +2566,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>W1580X</t>
+          <t>TN1020</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>LaserJet Tank 1020, 2506, LaserJet Neverstop / Tank 1005, LaserJet Tank 2606</t>
+          <t>HL-1111, HL-1201, HL-1211W, DCP-1511, DCP-1514, DCP-1601, DCP-1616NW, MFC-1811, MFC-1814, MFC-1911NW</t>
         </is>
       </c>
     </row>
@@ -2582,17 +2586,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>CF325X</t>
+          <t>TN2150</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>LaserJet Enterprise M800, M806, M806dn, LaserJet Enterprise MFP M830z</t>
+          <t>DCP-7030, DCP-7040, DCP-7045N, HL-2140, HL-2025, HL-2150N, HL-2170W, MFC-7440N, MFC-7840W, MFC-7340, MFC-7345DN, MFC-7320, MFC-7345N</t>
         </is>
       </c>
     </row>
@@ -2602,17 +2606,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>CF289A</t>
+          <t>TN3185</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>LaserJet Enterprise M507</t>
+          <t>HL-5240, HL-5250, HL-5270, MFC-8460, MFC-8860</t>
         </is>
       </c>
     </row>
@@ -2622,17 +2626,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>CE390X</t>
+          <t>TN3350</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>LaserJet P4014, P4015, P4515, LaserJet Enterprise M601, M602, M603, M4555</t>
+          <t>HL-5440, DCP-8110DN, DCP-8150DN, DCP-8250DN, MFC-8510DN, MFC-8910DW, HL-5450DN, HL-5470DW, HL-6180DW, MFC-8520DN, MFC-8710DW, MFC-8950DW</t>
         </is>
       </c>
     </row>
@@ -2642,17 +2646,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>CE390A</t>
+          <t>TN3448</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>LaserJet P4014, P4015, P4515, LaserJet Enterprise M601, M602, M603, M4555</t>
+          <t>HL-L5000D, HL-L5100DN, HL-L5200DW, HL-L6200DW, HL-L6400DW, MFC-L5700DN, MFC-L5800DW, MFC-L5900DW, MFC-L6700DW, MFC-L6900DW</t>
         </is>
       </c>
     </row>
@@ -2662,17 +2666,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>W1004AC</t>
+          <t>TN3478</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Laser MFP 131a, Laser 103a</t>
+          <t>HL-L5000D, HL-L5100DN, HL-L5200DW, HL-L6200DW, HL-L6400DW, MFC-L5700DN, MFC-L5800DW, MFC-L5900DW, MFC-L6700DW, MFC-L6900DW</t>
         </is>
       </c>
     </row>
@@ -2682,17 +2686,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>W1335X</t>
+          <t>TN2465</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>LaserJet MFP M438, M442dn, M443</t>
+          <t>HL-L2310D, HL-L2350DW, HL-L2370DN, DCP-L2510D, DCP-L2530DW, MFC-L2710DW, MFC-L2750DW</t>
         </is>
       </c>
     </row>
@@ -2702,17 +2706,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>W1370X</t>
+          <t>TN261BK/TN261C/TN261Y/TN261M</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>LaserJet M208, M209, M211d, LaserJet MFP M232, M233, M234, M236</t>
+          <t>HL-3140CW, HL-3150CDN, HL-3150CDW, HL-3170CDW, MFC-9130CW, MFC-9140CDN, MFC-9330CDW, MFC-9340CDW</t>
         </is>
       </c>
     </row>
@@ -2722,17 +2726,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>CE320A/CE321A/CE322A/CE323A</t>
+          <t>TN267BK/TN267C/TN267Y/TN267M</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Color LaserJet CP1525, CM1415, Color LaserJet Pro 200</t>
+          <t>HL-L3230CDN, MFC-L3750</t>
         </is>
       </c>
     </row>
@@ -2742,17 +2746,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CF210A/CF211A/CF212A/CF213A</t>
+          <t>TN2060</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro 200</t>
+          <t>HL-2130, HL-2132, DCP-7055, DCP-7057</t>
         </is>
       </c>
     </row>
@@ -2762,17 +2766,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>CF350A/CF351A/CF352A/CF353A</t>
+          <t>TN3280</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>HP / Canon</t>
+          <t>Brother</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>HP Color LaserJet Pro MFP M176 / Canon LBP7018C</t>
+          <t>HL-5340D, HL-5350DN, HL-5370DW, HL-5380DN, MFC-8370, MFC-8380DN, MFC-8480, MFC-8680, MFC-8690, MFC-8880DN, MFC-8890, DCP-8070, DCP-8085</t>
         </is>
       </c>
     </row>
@@ -2782,17 +2786,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>CE410A/CE411A/CE412A/CE413A</t>
+          <t>MLT-D111S</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro 300 M351, Color LaserJet Pro 300 MFP M375nw, Color LaserJet Pro 400 M451nw, M451dn, M451dw, Color LaserJet Pro 400 MFP M475dn, M475dw</t>
+          <t>Xpress SL-M2020, SL-M2020W, SL-M2021, SL-M2021W, SL-M2022, SL-M2022W, SL-M2024, SL-M2026, SL-M2026W, SL-M2070, SL-M2070W, SL-M2070F, SL-M2070FW, SL-M2071, SL-M2071W, SL-M2071FH, SL-M2074FW, SL-M2077, SL-M2078, SL-M2078F, SL-M2078FW</t>
         </is>
       </c>
     </row>
@@ -2802,17 +2806,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CF380A/CF381A/CF382A/CF383A</t>
+          <t>CLT-K404S/CLT-C404S/CLT-Y404S/CLT-M404S</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro MFP M476dn</t>
+          <t>Xpress SL-C430, SL-C432W, SL-C432, SL-C433W, SL-C433, SL-C480, SL-C480FN, SL-C480FW, SL-C480W, SL-C482, SL-C482FW, SL-C482W, SL-C483, SL-C483W, SL-C483FW</t>
         </is>
       </c>
     </row>
@@ -2822,17 +2826,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>CF500A/CF501A/CF502A/CF503A</t>
+          <t>MLT-D101</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro M254, Color LaserJet Pro MFP M280, M281</t>
+          <t>ML-2161, SCX-3401, SCX-3046, SF-760P, ML-2166</t>
         </is>
       </c>
     </row>
@@ -2842,17 +2846,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Q6000A/Q6001A/Q6002A/Q6003A</t>
+          <t>MLT-D103</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Color LaserJet 1600, 2600n, 2605, 2605dn, 2605dtn, CM1017, CM1015</t>
+          <t>ML-2951NDR, ML-2956DW, SCX-4701ND, SCX-4727FD, SCX-4728FD, SCX-4729FW</t>
         </is>
       </c>
     </row>
@@ -2862,17 +2866,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>CE250A/CE251A/CE252A/CE253A</t>
+          <t>MLT-D109</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Color LaserJet CP3525, CP3525n, CP3525dn, CM3530, CM3530fs</t>
+          <t>SCX-4300, SCX-4310, SCX-4315</t>
         </is>
       </c>
     </row>
@@ -2882,17 +2886,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>CE400A/CE401A/CE402A/CE403A</t>
+          <t>MLT-D110</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Color LaserJet Enterprise 500 M551n, M551dn, M551xh</t>
+          <t>Xpress SL-M2060</t>
         </is>
       </c>
     </row>
@@ -2902,17 +2906,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CE260A/CE261A/CE262A/CE263A</t>
+          <t>MLT-D115</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Color LaserJet CP4025, CP4520, CM4540</t>
+          <t>Xpress SL-M2620, SL-M2670, SL-M2820, SL-M2830</t>
         </is>
       </c>
     </row>
@@ -2922,17 +2926,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>CE270A/CE271A/CE272A/CE273A</t>
+          <t>MLT-D116</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Color LaserJet CP5525n, CP5525dn, CP5525xh</t>
+          <t>Xpress SL-M2625, SL-M2626, SL-M2825, SL-M2826, SL-M2675, SL-M2676, SL-M2875, SL-M2876</t>
         </is>
       </c>
     </row>
@@ -2942,17 +2946,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>W2310A/W2311A/W2312A/W2313A</t>
+          <t>MLT-D117</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro M155, Color LaserJet Pro MFP M182, M183</t>
+          <t>SCX-4021S, SCX-4650, SCX-4655F</t>
         </is>
       </c>
     </row>
@@ -2962,17 +2966,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>W2040A/W2041A/W2042A/W2043A</t>
+          <t>MLT-D203L</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Color LaserJet Pro M454, Color LaserJet Pro MFP M479</t>
+          <t>ProXpress SL-M3320, SL-M3820, SL-M4020, SL-M3370, SL-M3870, SL-M4070</t>
         </is>
       </c>
     </row>
@@ -2982,17 +2986,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>W2090A/W2091A/W2092A/W2093A</t>
+          <t>MLT-D203E</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Color Laser MFP 178nw, Color Laser 150a, 150nw</t>
+          <t>ProXpress SL-M3820, SL-M4020, SL-M3870, SL-M4070</t>
         </is>
       </c>
     </row>
@@ -3002,17 +3006,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>CE740A/CE741A/CE742A/CE743A</t>
+          <t>MLT-D205L</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Color LaserJet CP5225, CP5225n, CP5225dn</t>
+          <t>ML-3310, ML-3710, SCX-4833, SCX-5637, SCX-5639, SCX-5737</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3026,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>CLT-K404S/CLT-C404S/CLT-Y404S/CLT-M404S</t>
+          <t>MLT-D707</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3032,7 +3036,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Xpress SL-C430, SL-C432W, SL-C432, SL-C433W, SL-C433, SL-C480, SL-C480FN, SL-C480FW, SL-C480W, SL-C482, SL-C482FW, SL-C482W, SL-C483, SL-C483W, SL-C483FW</t>
+          <t>Xpress SL-K2200, SL-K2200ND</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3046,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>MLT-D101</t>
+          <t>MLT-D1043</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3052,7 +3056,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>ML-2161, SCX-3401, SCX-3046, SF-760P, ML-2166</t>
+          <t>ML-1666, SCX-3201, ML-1866, SCX-3206</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3066,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>MLT-D103</t>
+          <t>MLT-D1053</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3072,7 +3076,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>ML-2951NDR, ML-2956DW, SCX-4701ND, SCX-4727FD, SCX-4728FD, SCX-4729FW</t>
+          <t>ML-1911, ML-2526, SCX-4601, SCX-4623</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3086,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>MLT-D109</t>
+          <t>MLT-D108</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3092,7 +3096,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>SCX-4300, SCX-4310, SCX-4315</t>
+          <t>ML-1640, ML-1641, ML-2240, ML-2241</t>
         </is>
       </c>
     </row>
@@ -3102,17 +3106,17 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>MLT-D110</t>
+          <t>ML-1610</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung / Xerox</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Xpress SL-M2060</t>
+          <t>Samsung ML-1610, ML-1615, ML-2010, ML-2510 / Xerox Phaser 3117, Phaser 3122</t>
         </is>
       </c>
     </row>
@@ -3122,17 +3126,17 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>MLT-D115</t>
+          <t>ML-1710</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung / Xerox</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Xpress SL-M2620, SL-M2670, SL-M2820, SL-M2830</t>
+          <t>Samsung ML-1710, ML-1750, SCX-4016, SCX-4100, SCX-4216 / Xerox WorkCentre PE16, WorkCentre PE114, Phaser 3115</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3146,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>MLT-D116</t>
+          <t>ML-D2850</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3152,7 +3156,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Xpress SL-M2625, SL-M2626, SL-M2825, SL-M2826, SL-M2675, SL-M2676, SL-M2875, SL-M2876</t>
+          <t>ML-2850, ML-2851, ML-2855</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3166,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>MLT-D117</t>
+          <t>SCX-4200</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3172,7 +3176,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>SCX-4021S, SCX-4650, SCX-4655F</t>
+          <t>SCX-4200, ML-4200</t>
         </is>
       </c>
     </row>
@@ -3182,7 +3186,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>MLT-D203L</t>
+          <t>4725</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3192,7 +3196,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>ProXpress SL-M3320, SL-M3820, SL-M4020, SL-M3370, SL-M3870, SL-M4070</t>
+          <t>ML-4521F, ML-4321, ML-4521HS</t>
         </is>
       </c>
     </row>
@@ -3202,17 +3206,17 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>MLT-D203E</t>
+          <t>TK-160</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>ProXpress SL-M3820, SL-M4020, SL-M3870, SL-M4070</t>
+          <t>FS-1120D, FS-1120DN, ECOSYS P2035d, P2035dn</t>
         </is>
       </c>
     </row>
@@ -3222,17 +3226,17 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>MLT-D205L</t>
+          <t>TK-1122</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>ML-3310, ML-4833</t>
+          <t>FS-1060DN, FS-1025MFP, FS-1125MFP</t>
         </is>
       </c>
     </row>
@@ -3242,17 +3246,17 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>MLT-D707</t>
+          <t>TK-1134</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Xpress SL-K2200, SL-K2200ND</t>
+          <t>FS-1030MFP, FS-1130MFP, ECOSYS M2030dn, M2530dn</t>
         </is>
       </c>
     </row>
@@ -3262,17 +3266,17 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>MLT-D1043</t>
+          <t>TK-1140</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>ML-1666, SCX-3201, ML-1866, SCX-3206</t>
+          <t>FS-1035MFP, FS-1135MFP, ECOSYS M2035dn, M2535dn</t>
         </is>
       </c>
     </row>
@@ -3282,17 +3286,17 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>MLT-D1053</t>
+          <t>TK-1144</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ML-1911, ML-2526, SCX-4601, SCX-4623</t>
+          <t>FS-1035MFP, FS-1135MFP, ECOSYS M2035dn, M2535dn</t>
         </is>
       </c>
     </row>
@@ -3302,17 +3306,17 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>MLT-D108</t>
+          <t>TK-1170</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>ML-1640, ML-1641, ML-2240, ML-2241</t>
+          <t>ECOSYS M2040dn, M2540dn, M2640idw</t>
         </is>
       </c>
     </row>
@@ -3322,17 +3326,17 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>ML-1610</t>
+          <t>TK-3100</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Samsung / Xerox</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Samsung ML-1610, ML-2010, ML-2510, ML-4521, ML-4321 / Xerox Phaser 3117, 3122</t>
+          <t>FS-2100D, FS-2100DN, FS-4100DN, FS-4200DN, FS-4300DN, ECOSYS M3040dn, M3540dn</t>
         </is>
       </c>
     </row>
@@ -3342,17 +3346,17 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>ML-1710</t>
+          <t>TK-410</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Samsung / Xerox</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Samsung ML-1710, ML-1750, SCX-4016, SCX-4100, SCX-4216 / Xerox WorkCentre PE16, PE114, Phaser 3115</t>
+          <t>KM-1620, KM-1635, KM-1650, KM-2020, KM-2050, KM-2250</t>
         </is>
       </c>
     </row>
@@ -3362,17 +3366,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>ML-D2850</t>
+          <t>TK-4109</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>ML-2850, ML-2851, ML-2855</t>
+          <t>TASKalfa 1800, 2200</t>
         </is>
       </c>
     </row>
@@ -3382,17 +3386,17 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>SCX-4200</t>
+          <t>TK-1178</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>SCX-4200, ML-4200</t>
+          <t>ECOSYS M2040dn, M2540dn</t>
         </is>
       </c>
     </row>
@@ -3402,17 +3406,17 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>4725</t>
+          <t>TK-1114</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>ML-4521F, ML-4321, ML-4521HS</t>
+          <t>FS-1020, FS-1040, FS-1020MFP, FS-1120MFP</t>
         </is>
       </c>
     </row>
@@ -3422,17 +3426,17 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>1025</t>
+          <t>TK-1158</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Xerox</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>B1022, B1025</t>
+          <t>ECOSYS P2235</t>
         </is>
       </c>
     </row>
@@ -3442,17 +3446,17 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>TK-1168</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Xerox</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>B205, B210, B215</t>
+          <t>ECOSYS P2040dn, P2040dw</t>
         </is>
       </c>
     </row>
@@ -3462,17 +3466,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>3250</t>
+          <t>TK-7120</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Xerox</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Phaser 3250</t>
+          <t>TASKalfa 3212i</t>
         </is>
       </c>
     </row>
@@ -3482,17 +3486,17 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>3225</t>
+          <t>TK-3165</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Xerox</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Phaser 3052, 3260, WorkCentre 3215, 3225</t>
+          <t>ECOSYS P3050dn, P3055dn, P3060dn</t>
         </is>
       </c>
     </row>
@@ -3502,17 +3506,17 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>3025</t>
+          <t>TK-1148</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Xerox</t>
+          <t>Kyocera</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>WorkCentre 3025, Phaser 3020</t>
+          <t>ECOSYS M2135dn, M2635dn, M2735dw, P2235dn, P2235dw</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3526,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>5019</t>
+          <t>1025</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -3532,7 +3536,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>WorkCentre 5019, 5021</t>
+          <t>B1022, B1025</t>
         </is>
       </c>
     </row>
@@ -3542,17 +3546,17 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>KX-FAT410</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Xerox</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>KX-MB1500, KX-MB1520, KX-MB1503, KX-MB1508, KX-MB1530</t>
+          <t>B205, B210, B215</t>
         </is>
       </c>
     </row>
@@ -3562,17 +3566,17 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>SP100</t>
+          <t>3250</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Ricoh</t>
+          <t>Xerox</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>SP 100, 111</t>
+          <t>Phaser 3250</t>
         </is>
       </c>
     </row>
@@ -3582,17 +3586,17 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>SP200</t>
+          <t>3225</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Ricoh</t>
+          <t>Xerox</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>SP 200, 202, 203, 204S, 211, 213, 210, 212</t>
+          <t>Phaser 3052, 3260, WorkCentre 3215, 3225</t>
         </is>
       </c>
     </row>
@@ -3602,17 +3606,17 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>SP300</t>
+          <t>3025</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Ricoh</t>
+          <t>Xerox</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>SP 300</t>
+          <t>WorkCentre 3025, Phaser 3020</t>
         </is>
       </c>
     </row>
@@ -3622,17 +3626,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>SP310</t>
+          <t>5019</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Ricoh</t>
+          <t>Xerox</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>SP 310, 311, 312, 325, 320</t>
+          <t>WorkCentre 5019, 5021</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3646,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>SP3510</t>
+          <t>SP100</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3652,7 +3656,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>SP 3400, 3410, 3510, 3500</t>
+          <t>SP 100, 111</t>
         </is>
       </c>
     </row>
@@ -3662,7 +3666,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>1230D</t>
+          <t>SP200</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -3672,7 +3676,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1230D, Aficio MP1610LD, MP1610L, 2020D, 2015L, 2018D, 2018, 2015, 2000</t>
+          <t>SP 200, 202, 203, 204S, 211, 213, 210, 212</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3686,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2501</t>
+          <t>SP300</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -3692,7 +3696,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>2501, MP 2001L</t>
+          <t>SP 300</t>
         </is>
       </c>
     </row>
@@ -3702,17 +3706,17 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>503</t>
+          <t>SP310</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Lexmark</t>
+          <t>Ricoh</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>MS310, MS410d, MS510dn, MS610de, MS610dn, MS610dte, MS610dtn</t>
+          <t>SP 310, 311, 312, 325, 320</t>
         </is>
       </c>
     </row>
@@ -3722,17 +3726,17 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>T-1810D</t>
+          <t>SP3510</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Toshiba</t>
+          <t>Ricoh</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>e-STUDIO 181, 182, 211, 212, 242</t>
+          <t>SP 3400, 3410, 3510, 3500</t>
         </is>
       </c>
     </row>
@@ -3742,17 +3746,17 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>TK-410</t>
+          <t>1230D</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>Ricoh</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>KM-1620, KM-1635, KM-1650, KM-2020, KM-2050, KM-2250</t>
+          <t>1230D, Aficio MP1610LD, MP1610L, 2020D, 2015L, 2018D, 2018, 2015, 2000</t>
         </is>
       </c>
     </row>
@@ -3762,17 +3766,17 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>TK-4109</t>
+          <t>2501</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>Ricoh</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>TASKalfa 1800, 2200</t>
+          <t>2501, MP 2001L</t>
         </is>
       </c>
     </row>
@@ -3782,17 +3786,17 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>TK-1178</t>
+          <t>PC-210</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>Pantum</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>ECOSYS M2040dn, M2540dn</t>
+          <t>P2200, P2207, P2500, M6500, M6550</t>
         </is>
       </c>
     </row>
@@ -3802,17 +3806,17 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>TK-1114</t>
+          <t>PC-208</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>Pantum</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>FS-1020, FS-1040</t>
+          <t>P2508, M6508, M6558</t>
         </is>
       </c>
     </row>
@@ -3822,17 +3826,17 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>TK-1158</t>
+          <t>TL-412</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>Pantum</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>ECOSYS P2235</t>
+          <t>BP5100, BM5100</t>
         </is>
       </c>
     </row>
@@ -3842,17 +3846,17 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>TK-1168</t>
+          <t>TL-425</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>Pantum</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>ECOSYS P2235dn, P2235dw, P2040dn, P2040dw, M2135dn, M2635dn, M2735dw</t>
+          <t>BP5100DN, BM5100ADN</t>
         </is>
       </c>
     </row>
@@ -3862,17 +3866,17 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>TK-7120</t>
+          <t>TL-5120</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Kyocera</t>
+          <t>Pantum</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>TASKalfa 3212i</t>
+          <t>BP5100 series, BM5100 series</t>
         </is>
       </c>
     </row>
@@ -3882,15 +3886,19 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>TK-3165</t>
+          <t>PC-210KEV</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Kyocera</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr"/>
+          <t>Pantum</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>P2200</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -3898,7 +3906,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>PC-210KEV</t>
+          <t>PC-211KEV</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3908,7 +3916,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>P2200</t>
+          <t>P2500</t>
         </is>
       </c>
     </row>
@@ -3918,7 +3926,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>PC-211KEV</t>
+          <t>PC-310K</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -3928,7 +3936,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>P2500</t>
+          <t>P3500</t>
         </is>
       </c>
     </row>
@@ -3938,7 +3946,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>PC-310K</t>
+          <t>PC-310XK</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -3958,7 +3966,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>PC-310XK</t>
+          <t>TL-412K</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -3968,7 +3976,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>P3500</t>
+          <t>P3302, M7102</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3986,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>TL-412K</t>
+          <t>TL-412HK</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -3988,7 +3996,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>P3302, M7102</t>
+          <t>P3300, M7102</t>
         </is>
       </c>
     </row>
@@ -3998,7 +4006,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>TL-412HK</t>
+          <t>TL-412XK</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4018,17 +4026,77 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>TL-412XK</t>
+          <t>1130</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Pantum</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>P3300, M7102</t>
+          <t>Dell 1130</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>179</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>503</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Lexmark</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>MS310, MS410d, MS510dn, MS610de, MS610dn, MS610dte, MS610dtn</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>180</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>KX-FAT410</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>KX-MB1500, KX-MB1520, KX-MB1503, KX-MB1508, KX-MB1530</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>181</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>T-1810D</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Toshiba</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>e-STUDIO 181, 182, 211, 212, 242</t>
         </is>
       </c>
     </row>

</xml_diff>